<commit_message>
Review fixes: clearer rules, 4th example, layout examples, friendlier errors (v3)
</commit_message>
<xml_diff>
--- a/incident_reports.xlsx
+++ b/incident_reports.xlsx
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Weekly test: the emergency shower in Lab 3 gave only a weak trickle, far below the required flow; tagged out of use until repaired.</t>
+          <t>Weekly test: the emergency shower in Lab 3 gave almost no water, far below the required flow; tagged out of use until repaired.</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Weekly test: the eyewash station in pilot plant bay A gave only a weak trickle, far below the required flow; tagged out of use until repaired.</t>
+          <t>Weekly test: the eyewash station in pilot plant bay A gave almost no water, far below the required flow; tagged out of use until repaired.</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Weekly test: the emergency shower in Lab 1 gave only a weak trickle, far below the required flow; tagged out of use until repaired.</t>
+          <t>Weekly test: the emergency shower in Lab 1 gave almost no water, far below the required flow; tagged out of use until repaired.</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Weekly test: the eyewash station in Lab 3 gave only a weak trickle, far below the required flow; tagged out of use until repaired.</t>
+          <t>Weekly test: the eyewash station in Lab 3 gave almost no water, far below the required flow; tagged out of use until repaired.</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Weekly test: the eyewash station in Lab 2 gave only a weak trickle, far below the required flow; tagged out of use until repaired.</t>
+          <t>Weekly test: the eyewash station in Lab 2 gave almost no water, far below the required flow; tagged out of use until repaired.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Weekly test: the emergency shower in pilot plant bay B gave only a weak trickle, far below the required flow; tagged out of use until repaired.</t>
+          <t>Weekly test: the emergency shower in pilot plant bay B gave almost no water, far below the required flow; tagged out of use until repaired.</t>
         </is>
       </c>
     </row>

</xml_diff>